<commit_message>
feat: add scenario and source exports
</commit_message>
<xml_diff>
--- a/llm-hardware-estimator/outputs/qwen32b_compare.xlsx
+++ b/llm-hardware-estimator/outputs/qwen32b_compare.xlsx
@@ -5,8 +5,10 @@
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="GPU_Comparison" sheetId="2" r:id="rId2"/>
     <sheet name="Precision_Comparison" sheetId="3" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" r:id="rId4"/>
-    <sheet name="Validation" sheetId="5" r:id="rId5"/>
+    <sheet name="Scenario_Comparison" sheetId="4" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="5" r:id="rId5"/>
+    <sheet name="Sources" sheetId="6" r:id="rId6"/>
+    <sheet name="Validation" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -775,170 +777,280 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>scenario</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>required_memory_gb</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>production_memory_gb</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>suggested_gpu_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>suggested_gpu_memory_gb</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>suggested_gpu_model</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>rag</t>
+          <t>chat</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1024</v>
+      </c>
+      <c r="C2">
+        <v>512</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>66.42760925292968</v>
+      </c>
+      <c r="F2">
+        <v>86.3558920288086</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>64.0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>input_tokens</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="B3">
-        <v>4096</v>
+        <v>2048</v>
+      </c>
+      <c r="C3">
+        <v>256</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>66.21198425292968</v>
+      </c>
+      <c r="F3">
+        <v>86.07557952880859</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>64.0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>output_tokens</t>
+          <t>embedding</t>
         </is>
       </c>
       <c r="B4">
-        <v>512</v>
+        <v>1024</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <v>70.16510925292968</v>
+      </c>
+      <c r="F4">
+        <v>91.21464202880858</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>64.0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>concurrency</t>
+          <t>long_doc</t>
         </is>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>32768</v>
+      </c>
+      <c r="C5">
+        <v>1024</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>84.54010925292968</v>
+      </c>
+      <c r="F5">
+        <v>109.90214202880858</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
+        <v>64.0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>weight_precision</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>bf16</t>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>4096</v>
+      </c>
+      <c r="C6">
+        <v>512</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>70.74010925292968</v>
+      </c>
+      <c r="F6">
+        <v>91.9621420288086</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>64.0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>activation_precision</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>bf16</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>kv_cache_precision</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>bf16</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>quantization</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>kv_cache_mode</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>gpu_utilization_target</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>runtime_overhead</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>{'absolute_gb': 2.0, 'weight_ratio': 0.1, 'kv_cache_ratio': 0.15}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>production_margin_ratio</t>
-        </is>
-      </c>
-      <c r="B13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>parallel</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>{'strategy': 'none', 'tensor_parallel_size': 1, 'pipeline_parallel_size': 1, 'parallel_overhead_factor': 1.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>decision_goal</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>balanced</t>
+          <t>reranker</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>1024</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>67.86510925292968</v>
+      </c>
+      <c r="F7">
+        <v>88.22464202880859</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>64.0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>可作为生产试点</t>
         </is>
       </c>
     </row>
@@ -949,6 +1061,412 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>weight_precision</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>activation_precision</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>kv_cache_precision</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>quantization</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>kv_cache_mode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>gpu_utilization_target</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>runtime_overhead</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>{'absolute_gb': 2.0, 'weight_ratio': 0.1, 'kv_cache_ratio': 0.15}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>production_margin_ratio</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>parallel</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>{'strategy': 'none', 'tensor_parallel_size': 1, 'pipeline_parallel_size': 1, 'parallel_overhead_factor': 1.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>decision_goal</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>hardware_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>gpu_model</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>last_checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>muxi-c500-64g</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>沐曦</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>曦云C500 64GB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>software_official_hardware_third_party</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://lmdeploy.readthedocs.io/zh-cn/latest/get_started/maca/get_started.html</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ascend-910b-64g</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>华为昇腾</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>910B 64GB平台</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>official_plus_supplier</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://e.huawei.com/cn/products/computing/ascend/atlas-800i-a2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mthreads-s4000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>摩尔线程</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MTT S4000</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://docs.mthreads.com/s4000/s4000-doc-online/product_specifications/</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cambricon-mlu370-x8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>寒武纪</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MLU370-X8</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://cambricon.com/index.php?a=lists&amp;c=index&amp;catid=406&amp;m=content</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>kunlunxin-r200-32g</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>昆仑芯</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>R200-8F 32GB</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.kunlunxin.com/product/274.html</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
     <row r="1"/>
   </sheetData>
 </worksheet>

</xml_diff>